<commit_message>
:bat: diversity stat without Mothers_0days
</commit_message>
<xml_diff>
--- a/data/derived_data/4_Diversities/ps_ITS_rare_expe_D1_mtd_table.xlsx
+++ b/data/derived_data/4_Diversities/ps_ITS_rare_expe_D1_mtd_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -486,6 +486,9 @@
   </si>
   <si>
     <t xml:space="preserve">MS_155</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS_156</t>
   </si>
   <si>
     <t xml:space="preserve">MS_157</t>
@@ -6567,7 +6570,7 @@
         <v>146</v>
       </c>
       <c r="E97" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="F97" t="s">
         <v>147</v>
@@ -6585,19 +6588,19 @@
         <v>45</v>
       </c>
       <c r="K97" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="L97" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M97" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N97" t="s">
         <v>25</v>
       </c>
       <c r="O97" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="P97" t="s">
         <v>31</v>
@@ -6656,7 +6659,7 @@
         <v>25</v>
       </c>
       <c r="O98" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P98" t="s">
         <v>31</v>
@@ -6715,7 +6718,7 @@
         <v>25</v>
       </c>
       <c r="O99" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P99" t="s">
         <v>31</v>
@@ -6744,7 +6747,7 @@
         <v>146</v>
       </c>
       <c r="E100" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="F100" t="s">
         <v>147</v>
@@ -6753,28 +6756,28 @@
         <v>60</v>
       </c>
       <c r="H100" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="I100" t="s">
         <v>26</v>
       </c>
       <c r="J100" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="K100" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="L100" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="M100" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="N100" t="s">
         <v>25</v>
       </c>
       <c r="O100" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="P100" t="s">
         <v>31</v>
@@ -6833,7 +6836,7 @@
         <v>25</v>
       </c>
       <c r="O101" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P101" t="s">
         <v>31</v>
@@ -6862,7 +6865,7 @@
         <v>146</v>
       </c>
       <c r="E102" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="F102" t="s">
         <v>147</v>
@@ -6892,7 +6895,7 @@
         <v>25</v>
       </c>
       <c r="O102" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P102" t="s">
         <v>31</v>
@@ -6936,22 +6939,22 @@
         <v>26</v>
       </c>
       <c r="J103" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="K103" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L103" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="M103" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="N103" t="s">
         <v>25</v>
       </c>
       <c r="O103" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="P103" t="s">
         <v>31</v>
@@ -7010,7 +7013,7 @@
         <v>25</v>
       </c>
       <c r="O104" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P104" t="s">
         <v>31</v>
@@ -7039,7 +7042,7 @@
         <v>146</v>
       </c>
       <c r="E105" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="F105" t="s">
         <v>147</v>
@@ -7069,7 +7072,7 @@
         <v>25</v>
       </c>
       <c r="O105" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P105" t="s">
         <v>31</v>
@@ -7098,7 +7101,7 @@
         <v>146</v>
       </c>
       <c r="E106" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F106" t="s">
         <v>147</v>
@@ -7119,16 +7122,16 @@
         <v>36</v>
       </c>
       <c r="L106" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="M106" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="N106" t="s">
         <v>25</v>
       </c>
       <c r="O106" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="P106" t="s">
         <v>31</v>
@@ -7157,7 +7160,7 @@
         <v>146</v>
       </c>
       <c r="E107" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="F107" t="s">
         <v>147</v>
@@ -7187,7 +7190,7 @@
         <v>25</v>
       </c>
       <c r="O107" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P107" t="s">
         <v>31</v>
@@ -7216,7 +7219,7 @@
         <v>146</v>
       </c>
       <c r="E108" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="F108" t="s">
         <v>147</v>
@@ -7231,22 +7234,22 @@
         <v>26</v>
       </c>
       <c r="J108" t="s">
+        <v>35</v>
+      </c>
+      <c r="K108" t="s">
+        <v>36</v>
+      </c>
+      <c r="L108" t="s">
+        <v>37</v>
+      </c>
+      <c r="M108" t="s">
+        <v>38</v>
+      </c>
+      <c r="N108" t="s">
+        <v>25</v>
+      </c>
+      <c r="O108" t="s">
         <v>45</v>
-      </c>
-      <c r="K108" t="s">
-        <v>46</v>
-      </c>
-      <c r="L108" t="s">
-        <v>47</v>
-      </c>
-      <c r="M108" t="s">
-        <v>48</v>
-      </c>
-      <c r="N108" t="s">
-        <v>25</v>
-      </c>
-      <c r="O108" t="s">
-        <v>27</v>
       </c>
       <c r="P108" t="s">
         <v>31</v>
@@ -7305,7 +7308,7 @@
         <v>25</v>
       </c>
       <c r="O109" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P109" t="s">
         <v>31</v>
@@ -7364,7 +7367,7 @@
         <v>25</v>
       </c>
       <c r="O110" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P110" t="s">
         <v>31</v>
@@ -7411,19 +7414,19 @@
         <v>45</v>
       </c>
       <c r="K111" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="L111" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M111" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N111" t="s">
         <v>25</v>
       </c>
       <c r="O111" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="P111" t="s">
         <v>31</v>
@@ -7482,7 +7485,7 @@
         <v>25</v>
       </c>
       <c r="O112" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P112" t="s">
         <v>31</v>
@@ -7511,7 +7514,7 @@
         <v>146</v>
       </c>
       <c r="E113" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="F113" t="s">
         <v>147</v>
@@ -7541,7 +7544,7 @@
         <v>25</v>
       </c>
       <c r="O113" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="P113" t="s">
         <v>31</v>
@@ -7564,52 +7567,52 @@
         <v>20</v>
       </c>
       <c r="C114" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D114" t="s">
-        <v>58</v>
+        <v>146</v>
       </c>
       <c r="E114" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F114" t="s">
-        <v>59</v>
+        <v>147</v>
       </c>
       <c r="G114" t="s">
         <v>60</v>
       </c>
       <c r="H114" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="I114" t="s">
         <v>26</v>
       </c>
       <c r="J114" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="K114" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="L114" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="M114" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="N114" t="s">
         <v>25</v>
       </c>
       <c r="O114" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="P114" t="s">
         <v>31</v>
       </c>
       <c r="Q114" t="s">
-        <v>59</v>
+        <v>148</v>
       </c>
       <c r="R114" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="S114" t="s">
         <v>175</v>
@@ -7644,16 +7647,16 @@
         <v>26</v>
       </c>
       <c r="J115" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="K115" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L115" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="M115" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="N115" t="s">
         <v>25</v>
@@ -7688,7 +7691,7 @@
         <v>58</v>
       </c>
       <c r="E116" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="F116" t="s">
         <v>59</v>
@@ -7703,16 +7706,16 @@
         <v>26</v>
       </c>
       <c r="J116" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K116" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="L116" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="M116" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="N116" t="s">
         <v>25</v>
@@ -7747,7 +7750,7 @@
         <v>58</v>
       </c>
       <c r="E117" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="F117" t="s">
         <v>59</v>
@@ -7765,13 +7768,13 @@
         <v>45</v>
       </c>
       <c r="K117" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="L117" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="M117" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N117" t="s">
         <v>25</v>
@@ -7806,7 +7809,7 @@
         <v>58</v>
       </c>
       <c r="E118" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="F118" t="s">
         <v>59</v>
@@ -7815,22 +7818,22 @@
         <v>60</v>
       </c>
       <c r="H118" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="I118" t="s">
         <v>26</v>
       </c>
       <c r="J118" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="K118" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="L118" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="M118" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="N118" t="s">
         <v>25</v>
@@ -7880,16 +7883,16 @@
         <v>26</v>
       </c>
       <c r="J119" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="K119" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="L119" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="M119" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="N119" t="s">
         <v>25</v>
@@ -7924,7 +7927,7 @@
         <v>58</v>
       </c>
       <c r="E120" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="F120" t="s">
         <v>59</v>
@@ -7939,16 +7942,16 @@
         <v>26</v>
       </c>
       <c r="J120" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="K120" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L120" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="M120" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="N120" t="s">
         <v>25</v>
@@ -7983,7 +7986,7 @@
         <v>58</v>
       </c>
       <c r="E121" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="F121" t="s">
         <v>59</v>
@@ -7998,16 +8001,16 @@
         <v>26</v>
       </c>
       <c r="J121" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K121" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="L121" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="M121" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="N121" t="s">
         <v>25</v>
@@ -8026,6 +8029,65 @@
       </c>
       <c r="S121" t="s">
         <v>182</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s">
+        <v>183</v>
+      </c>
+      <c r="B122" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122" t="s">
+        <v>20</v>
+      </c>
+      <c r="D122" t="s">
+        <v>58</v>
+      </c>
+      <c r="E122" t="s">
+        <v>22</v>
+      </c>
+      <c r="F122" t="s">
+        <v>59</v>
+      </c>
+      <c r="G122" t="s">
+        <v>60</v>
+      </c>
+      <c r="H122" t="s">
+        <v>70</v>
+      </c>
+      <c r="I122" t="s">
+        <v>26</v>
+      </c>
+      <c r="J122" t="s">
+        <v>45</v>
+      </c>
+      <c r="K122" t="s">
+        <v>52</v>
+      </c>
+      <c r="L122" t="s">
+        <v>53</v>
+      </c>
+      <c r="M122" t="s">
+        <v>54</v>
+      </c>
+      <c r="N122" t="s">
+        <v>25</v>
+      </c>
+      <c r="O122" t="s">
+        <v>25</v>
+      </c>
+      <c r="P122" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q122" t="s">
+        <v>59</v>
+      </c>
+      <c r="R122" t="s">
+        <v>59</v>
+      </c>
+      <c r="S122" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>